<commit_message>
Regenerate outputs from committed notebook
</commit_message>
<xml_diff>
--- a/data/team2_step2_corr_package.xlsx
+++ b/data/team2_step2_corr_package.xlsx
@@ -4930,7 +4930,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.09005407607642206</v>
+        <v>0.09005407607642242</v>
       </c>
     </row>
     <row r="8">
@@ -4940,7 +4940,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>47.99513650649764</v>
+        <v>47.99513650649745</v>
       </c>
     </row>
     <row r="9">
@@ -4950,7 +4950,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001493330992415892</v>
+        <v>0.00149333099241589</v>
       </c>
     </row>
     <row r="10">
@@ -4960,7 +4960,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>80.84833239095349</v>
+        <v>80.84833239095363</v>
       </c>
     </row>
     <row r="11">

</xml_diff>